<commit_message>
working on label printing directions
I'm sure there's occasional bugs in the code, but it generally seems to be working. Things left: mess around with the word template a little more to create directions/optimize.
</commit_message>
<xml_diff>
--- a/example-sample-labels.xlsx
+++ b/example-sample-labels.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wampleka\Documents\Projects\WWS-standard-methods\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wampleka\Documents\Projects\WWS-standard-methods\Templates\water-quality-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7BE0AB7-0F3D-4F9B-BA86-2865BCF6AD4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD803461-5D87-4D8D-8E27-39BC4324F2CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sample-DateTime" sheetId="21" state="visible" r:id="rId1"/>
@@ -24,12 +24,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Site</t>
   </si>
@@ -116,753 +127,6 @@
   </si>
   <si>
     <t>Sample Type</t>
-  </si>
-  <si>
-    <t>BDRK_R0006</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_1500</t>
-  </si>
-  <si>
-    <t>STA</t>
-  </si>
-  <si>
-    <t>IS</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>20260223</t>
-  </si>
-  <si>
-    <t>1500</t>
-  </si>
-  <si>
-    <t>BDRK_R0024</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_1700</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>1700</t>
-  </si>
-  <si>
-    <t>BDRK_R0019</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_1900</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>1900</t>
-  </si>
-  <si>
-    <t>BDRK_R0003</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_2100</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>2100</t>
-  </si>
-  <si>
-    <t>BDRK_R0012</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_2300</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>2300</t>
-  </si>
-  <si>
-    <t>BDRK_R0030</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0100</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>20260224</t>
-  </si>
-  <si>
-    <t>0100</t>
-  </si>
-  <si>
-    <t>BDRK_R0044</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0300</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>0300</t>
-  </si>
-  <si>
-    <t>BDRK_R0037</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0500</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>0500</t>
-  </si>
-  <si>
-    <t>BDRK_R0018</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0700</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>0700</t>
-  </si>
-  <si>
-    <t>BDRK_R0045</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0900</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>0900</t>
-  </si>
-  <si>
-    <t>BDRK_R0042</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1100</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>1100</t>
-  </si>
-  <si>
-    <t>BDRK_R0035</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1300</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>1300</t>
-  </si>
-  <si>
-    <t>BDRK_R0047</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1500</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>BDRK_R0022</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1700</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>BDRK_R0016</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1900</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>BDRK_R0001</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_2100</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>BDRK_R0002</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_2300</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>BDRK_R0036</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0100</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>20260225</t>
-  </si>
-  <si>
-    <t>BDRK_R0028</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0300</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>BDRK_R0014</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0500</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>BDRK_R0026</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0700</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>BDRK_R0050</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0900</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>BDRK_R0049</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_1100</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>BDRK_R0039</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_1300</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>BDRK_R0033</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_1700</t>
-  </si>
-  <si>
-    <t>COA</t>
-  </si>
-  <si>
-    <t>BDRK_R0005</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_1900</t>
-  </si>
-  <si>
-    <t>BDRK_R0025</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_2100</t>
-  </si>
-  <si>
-    <t>BDRK_R0009</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_2300</t>
-  </si>
-  <si>
-    <t>BDRK_R0052</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0100</t>
-  </si>
-  <si>
-    <t>BDRK_R0011</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0300</t>
-  </si>
-  <si>
-    <t>BDRK_R0040</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0500</t>
-  </si>
-  <si>
-    <t>BDRK_R0023</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0700</t>
-  </si>
-  <si>
-    <t>BDRK_R0017</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0900</t>
-  </si>
-  <si>
-    <t>BDRK_R0015</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1100</t>
-  </si>
-  <si>
-    <t>BDRK_R0032</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1300</t>
-  </si>
-  <si>
-    <t>BDRK_R0038</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1500</t>
-  </si>
-  <si>
-    <t>BDRK_R0021</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1700</t>
-  </si>
-  <si>
-    <t>BDRK_R0029</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1900</t>
-  </si>
-  <si>
-    <t>BDRK_R0043</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_2100</t>
-  </si>
-  <si>
-    <t>BDRK_R0048</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_2300</t>
-  </si>
-  <si>
-    <t>BDRK_R0020</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0100</t>
-  </si>
-  <si>
-    <t>BDRK_R0034</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0300</t>
-  </si>
-  <si>
-    <t>BDRK_R0010</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0500</t>
-  </si>
-  <si>
-    <t>BDRK_R0007</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0700</t>
-  </si>
-  <si>
-    <t>BDRK_R0008</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0900</t>
-  </si>
-  <si>
-    <t>BDRK_R0041</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_1100</t>
-  </si>
-  <si>
-    <t>BDRK_R0027</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_1300</t>
-  </si>
-  <si>
-    <t>BDRK_R0013</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_1500</t>
-  </si>
-  <si>
-    <t>BDRK_R0031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BDRK_LBLK_IS_ _ </t>
-  </si>
-  <si>
-    <t>LBLK</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>BDRK_R0004</t>
-  </si>
-  <si>
-    <t>BDRK_R0051</t>
-  </si>
-  <si>
-    <t>BDRK_R0046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BDRK_FBLK_IS_ _ </t>
-  </si>
-  <si>
-    <t>FBLK</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_2100_AQ</t>
-  </si>
-  <si>
-    <t>Aqualog</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_2300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_2100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_LBLK_IS_ _ _AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_1900_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_1500_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0700_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0900_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_2300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0500_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_2300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_1500_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0500_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1900_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0900_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0700_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_1900_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1700_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1700_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0700_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_1700_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_2100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0700_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_1300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1900_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_1700_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0500_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1500_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_1300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0500_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_1100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_2100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0900_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_FBLK_IS_ _ _AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1500_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_2300_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_1100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0900_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0100_AQ</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_2100_CN</t>
-  </si>
-  <si>
-    <t>Shimadzu</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_2300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_2100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_LBLK_IS_ _ _CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_1900_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_1500_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0700_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0900_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_2300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0500_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_2300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_1500_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0500_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1900_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0900_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0700_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_1900_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1700_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1700_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0700_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260223_1700_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_2100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0700_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_1300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1900_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260223_1700_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_0300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0500_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_1500_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_1300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0500_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260225_1100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_2100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_0900_CN</t>
-  </si>
-  <si>
-    <t>BDRK_FBLK_IS_ _ _CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260224_1500_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_2300_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_1100_CN</t>
-  </si>
-  <si>
-    <t>BDRK_STA_IS_20260225_0900_CN</t>
-  </si>
-  <si>
-    <t>BDRK_COA_IS_20260224_0100_CN</t>
   </si>
 </sst>
 </file>
@@ -1774,7 +1038,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>BDRK_R0006</t>
@@ -1814,7 +1078,7 @@
         </is>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>BDRK_R0024</t>
@@ -1854,7 +1118,7 @@
         </is>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>BDRK_R0019</t>
@@ -1894,7 +1158,7 @@
         </is>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="inlineStr">
         <is>
           <t>BDRK_R0003</t>
@@ -1934,7 +1198,7 @@
         </is>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" t="inlineStr">
         <is>
           <t>BDRK_R0012</t>
@@ -1974,7 +1238,7 @@
         </is>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="A7" t="inlineStr">
         <is>
           <t>BDRK_R0030</t>
@@ -2014,7 +1278,7 @@
         </is>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" t="inlineStr">
         <is>
           <t>BDRK_R0044</t>
@@ -2054,7 +1318,7 @@
         </is>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" t="inlineStr">
         <is>
           <t>BDRK_R0037</t>
@@ -2094,7 +1358,7 @@
         </is>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>BDRK_R0018</t>
@@ -2134,7 +1398,7 @@
         </is>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="A11" t="inlineStr">
         <is>
           <t>BDRK_R0045</t>
@@ -2174,7 +1438,7 @@
         </is>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12">
       <c r="A12" t="inlineStr">
         <is>
           <t>BDRK_R0042</t>
@@ -2214,7 +1478,7 @@
         </is>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13">
       <c r="A13" t="inlineStr">
         <is>
           <t>BDRK_R0035</t>
@@ -2254,7 +1518,7 @@
         </is>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14">
       <c r="A14" t="inlineStr">
         <is>
           <t>BDRK_R0047</t>
@@ -2294,7 +1558,7 @@
         </is>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15">
       <c r="A15" t="inlineStr">
         <is>
           <t>BDRK_R0022</t>
@@ -2334,7 +1598,7 @@
         </is>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16">
       <c r="A16" t="inlineStr">
         <is>
           <t>BDRK_R0016</t>
@@ -2374,7 +1638,7 @@
         </is>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17">
       <c r="A17" t="inlineStr">
         <is>
           <t>BDRK_R0001</t>
@@ -2414,7 +1678,7 @@
         </is>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18">
       <c r="A18" t="inlineStr">
         <is>
           <t>BDRK_R0002</t>
@@ -2454,7 +1718,7 @@
         </is>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19">
       <c r="A19" t="inlineStr">
         <is>
           <t>BDRK_R0036</t>
@@ -2494,7 +1758,7 @@
         </is>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20">
       <c r="A20" t="inlineStr">
         <is>
           <t>BDRK_R0028</t>
@@ -2534,7 +1798,7 @@
         </is>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21">
       <c r="A21" t="inlineStr">
         <is>
           <t>BDRK_R0014</t>
@@ -2574,7 +1838,7 @@
         </is>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22">
       <c r="A22" t="inlineStr">
         <is>
           <t>BDRK_R0026</t>
@@ -2614,7 +1878,7 @@
         </is>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23">
       <c r="A23" t="inlineStr">
         <is>
           <t>BDRK_R0050</t>
@@ -2654,7 +1918,7 @@
         </is>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24">
       <c r="A24" t="inlineStr">
         <is>
           <t>BDRK_R0049</t>
@@ -2694,7 +1958,7 @@
         </is>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25">
       <c r="A25" t="inlineStr">
         <is>
           <t>BDRK_R0039</t>
@@ -2734,7 +1998,7 @@
         </is>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26">
       <c r="A26" t="inlineStr">
         <is>
           <t>BDRK_R0033</t>
@@ -2774,7 +2038,7 @@
         </is>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27">
       <c r="A27" t="inlineStr">
         <is>
           <t>BDRK_R0005</t>
@@ -2814,7 +2078,7 @@
         </is>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28">
       <c r="A28" t="inlineStr">
         <is>
           <t>BDRK_R0025</t>
@@ -2854,7 +2118,7 @@
         </is>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29">
       <c r="A29" t="inlineStr">
         <is>
           <t>BDRK_R0009</t>
@@ -2894,7 +2158,7 @@
         </is>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30">
       <c r="A30" t="inlineStr">
         <is>
           <t>BDRK_R0052</t>
@@ -2934,7 +2198,7 @@
         </is>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31">
       <c r="A31" t="inlineStr">
         <is>
           <t>BDRK_R0011</t>
@@ -2974,7 +2238,7 @@
         </is>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32">
       <c r="A32" t="inlineStr">
         <is>
           <t>BDRK_R0040</t>
@@ -3014,7 +2278,7 @@
         </is>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33">
       <c r="A33" t="inlineStr">
         <is>
           <t>BDRK_R0023</t>
@@ -3054,7 +2318,7 @@
         </is>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34">
       <c r="A34" t="inlineStr">
         <is>
           <t>BDRK_R0017</t>
@@ -3094,7 +2358,7 @@
         </is>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35">
       <c r="A35" t="inlineStr">
         <is>
           <t>BDRK_R0015</t>
@@ -3134,7 +2398,7 @@
         </is>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36">
       <c r="A36" t="inlineStr">
         <is>
           <t>BDRK_R0032</t>
@@ -3174,7 +2438,7 @@
         </is>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37">
       <c r="A37" t="inlineStr">
         <is>
           <t>BDRK_R0038</t>
@@ -3214,7 +2478,7 @@
         </is>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38">
       <c r="A38" t="inlineStr">
         <is>
           <t>BDRK_R0021</t>
@@ -3254,7 +2518,7 @@
         </is>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39">
       <c r="A39" t="inlineStr">
         <is>
           <t>BDRK_R0029</t>
@@ -3294,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40">
       <c r="A40" t="inlineStr">
         <is>
           <t>BDRK_R0043</t>
@@ -3334,7 +2598,7 @@
         </is>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41">
       <c r="A41" t="inlineStr">
         <is>
           <t>BDRK_R0048</t>
@@ -3374,7 +2638,7 @@
         </is>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42">
       <c r="A42" t="inlineStr">
         <is>
           <t>BDRK_R0020</t>
@@ -3414,7 +2678,7 @@
         </is>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43">
       <c r="A43" t="inlineStr">
         <is>
           <t>BDRK_R0034</t>
@@ -3454,7 +2718,7 @@
         </is>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44">
       <c r="A44" t="inlineStr">
         <is>
           <t>BDRK_R0010</t>
@@ -3494,7 +2758,7 @@
         </is>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45">
       <c r="A45" t="inlineStr">
         <is>
           <t>BDRK_R0007</t>
@@ -3534,7 +2798,7 @@
         </is>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46">
       <c r="A46" t="inlineStr">
         <is>
           <t>BDRK_R0008</t>
@@ -3574,7 +2838,7 @@
         </is>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47">
       <c r="A47" t="inlineStr">
         <is>
           <t>BDRK_R0041</t>
@@ -3614,7 +2878,7 @@
         </is>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48">
       <c r="A48" t="inlineStr">
         <is>
           <t>BDRK_R0027</t>
@@ -3654,7 +2918,7 @@
         </is>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49">
       <c r="A49" t="inlineStr">
         <is>
           <t>BDRK_R0013</t>
@@ -3694,7 +2958,7 @@
         </is>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50">
       <c r="A50" t="inlineStr">
         <is>
           <t>BDRK_R0031</t>
@@ -3702,7 +2966,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3725,16 +2989,16 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>20260510</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1000</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
       <c r="A51" t="inlineStr">
         <is>
           <t>BDRK_R0004</t>
@@ -3742,7 +3006,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3765,16 +3029,16 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>20260510</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1000</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
       <c r="A52" t="inlineStr">
         <is>
           <t>BDRK_R0051</t>
@@ -3782,7 +3046,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3805,16 +3069,16 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>20260510</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1000</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
       <c r="A53" t="inlineStr">
         <is>
           <t>BDRK_R0046</t>
@@ -3822,7 +3086,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>BDRK_FBLK_IS_20260510_1000</t>
+          <t>BDRK_FBLK_IS______________</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3845,12 +3109,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>20260510</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -3960,7 +3224,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>BDRK_R0006</t>
@@ -3977,7 +3241,7 @@
         </is>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>BDRK_R0024</t>
@@ -3994,7 +3258,7 @@
         </is>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>BDRK_R0019</t>
@@ -4011,7 +3275,7 @@
         </is>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="inlineStr">
         <is>
           <t>BDRK_R0003</t>
@@ -4028,7 +3292,7 @@
         </is>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" t="inlineStr">
         <is>
           <t>BDRK_R0012</t>
@@ -4045,7 +3309,7 @@
         </is>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="A7" t="inlineStr">
         <is>
           <t>BDRK_R0030</t>
@@ -4062,7 +3326,7 @@
         </is>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" t="inlineStr">
         <is>
           <t>BDRK_R0044</t>
@@ -4079,7 +3343,7 @@
         </is>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" t="inlineStr">
         <is>
           <t>BDRK_R0037</t>
@@ -4096,7 +3360,7 @@
         </is>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>BDRK_R0018</t>
@@ -4113,7 +3377,7 @@
         </is>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="A11" t="inlineStr">
         <is>
           <t>BDRK_R0045</t>
@@ -4130,7 +3394,7 @@
         </is>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12">
       <c r="A12" t="inlineStr">
         <is>
           <t>BDRK_R0042</t>
@@ -4147,7 +3411,7 @@
         </is>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13">
       <c r="A13" t="inlineStr">
         <is>
           <t>BDRK_R0035</t>
@@ -4164,7 +3428,7 @@
         </is>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14">
       <c r="A14" t="inlineStr">
         <is>
           <t>BDRK_R0047</t>
@@ -4181,7 +3445,7 @@
         </is>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15">
       <c r="A15" t="inlineStr">
         <is>
           <t>BDRK_R0022</t>
@@ -4198,7 +3462,7 @@
         </is>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16">
       <c r="A16" t="inlineStr">
         <is>
           <t>BDRK_R0016</t>
@@ -4215,7 +3479,7 @@
         </is>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17">
       <c r="A17" t="inlineStr">
         <is>
           <t>BDRK_R0001</t>
@@ -4232,7 +3496,7 @@
         </is>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18">
       <c r="A18" t="inlineStr">
         <is>
           <t>BDRK_R0002</t>
@@ -4249,7 +3513,7 @@
         </is>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19">
       <c r="A19" t="inlineStr">
         <is>
           <t>BDRK_R0036</t>
@@ -4266,7 +3530,7 @@
         </is>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20">
       <c r="A20" t="inlineStr">
         <is>
           <t>BDRK_R0028</t>
@@ -4283,7 +3547,7 @@
         </is>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21">
       <c r="A21" t="inlineStr">
         <is>
           <t>BDRK_R0014</t>
@@ -4300,7 +3564,7 @@
         </is>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22">
       <c r="A22" t="inlineStr">
         <is>
           <t>BDRK_R0026</t>
@@ -4317,7 +3581,7 @@
         </is>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23">
       <c r="A23" t="inlineStr">
         <is>
           <t>BDRK_R0050</t>
@@ -4334,7 +3598,7 @@
         </is>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24">
       <c r="A24" t="inlineStr">
         <is>
           <t>BDRK_R0049</t>
@@ -4351,7 +3615,7 @@
         </is>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25">
       <c r="A25" t="inlineStr">
         <is>
           <t>BDRK_R0039</t>
@@ -4368,7 +3632,7 @@
         </is>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26">
       <c r="A26" t="inlineStr">
         <is>
           <t>BDRK_R0033</t>
@@ -4385,7 +3649,7 @@
         </is>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27">
       <c r="A27" t="inlineStr">
         <is>
           <t>BDRK_R0005</t>
@@ -4402,7 +3666,7 @@
         </is>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28">
       <c r="A28" t="inlineStr">
         <is>
           <t>BDRK_R0025</t>
@@ -4419,7 +3683,7 @@
         </is>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29">
       <c r="A29" t="inlineStr">
         <is>
           <t>BDRK_R0009</t>
@@ -4436,7 +3700,7 @@
         </is>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30">
       <c r="A30" t="inlineStr">
         <is>
           <t>BDRK_R0052</t>
@@ -4453,7 +3717,7 @@
         </is>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31">
       <c r="A31" t="inlineStr">
         <is>
           <t>BDRK_R0011</t>
@@ -4470,7 +3734,7 @@
         </is>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32">
       <c r="A32" t="inlineStr">
         <is>
           <t>BDRK_R0040</t>
@@ -4487,7 +3751,7 @@
         </is>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33">
       <c r="A33" t="inlineStr">
         <is>
           <t>BDRK_R0023</t>
@@ -4504,7 +3768,7 @@
         </is>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34">
       <c r="A34" t="inlineStr">
         <is>
           <t>BDRK_R0017</t>
@@ -4521,7 +3785,7 @@
         </is>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35">
       <c r="A35" t="inlineStr">
         <is>
           <t>BDRK_R0015</t>
@@ -4538,7 +3802,7 @@
         </is>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36">
       <c r="A36" t="inlineStr">
         <is>
           <t>BDRK_R0032</t>
@@ -4555,7 +3819,7 @@
         </is>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37">
       <c r="A37" t="inlineStr">
         <is>
           <t>BDRK_R0038</t>
@@ -4572,7 +3836,7 @@
         </is>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38">
       <c r="A38" t="inlineStr">
         <is>
           <t>BDRK_R0021</t>
@@ -4589,7 +3853,7 @@
         </is>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39">
       <c r="A39" t="inlineStr">
         <is>
           <t>BDRK_R0029</t>
@@ -4606,7 +3870,7 @@
         </is>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40">
       <c r="A40" t="inlineStr">
         <is>
           <t>BDRK_R0043</t>
@@ -4623,7 +3887,7 @@
         </is>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41">
       <c r="A41" t="inlineStr">
         <is>
           <t>BDRK_R0048</t>
@@ -4640,7 +3904,7 @@
         </is>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42">
       <c r="A42" t="inlineStr">
         <is>
           <t>BDRK_R0020</t>
@@ -4657,7 +3921,7 @@
         </is>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43">
       <c r="A43" t="inlineStr">
         <is>
           <t>BDRK_R0034</t>
@@ -4674,7 +3938,7 @@
         </is>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44">
       <c r="A44" t="inlineStr">
         <is>
           <t>BDRK_R0010</t>
@@ -4691,7 +3955,7 @@
         </is>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45">
       <c r="A45" t="inlineStr">
         <is>
           <t>BDRK_R0007</t>
@@ -4708,7 +3972,7 @@
         </is>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46">
       <c r="A46" t="inlineStr">
         <is>
           <t>BDRK_R0008</t>
@@ -4725,7 +3989,7 @@
         </is>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47">
       <c r="A47" t="inlineStr">
         <is>
           <t>BDRK_R0041</t>
@@ -4742,7 +4006,7 @@
         </is>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48">
       <c r="A48" t="inlineStr">
         <is>
           <t>BDRK_R0027</t>
@@ -4759,7 +4023,7 @@
         </is>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49">
       <c r="A49" t="inlineStr">
         <is>
           <t>BDRK_R0013</t>
@@ -4776,7 +4040,7 @@
         </is>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50">
       <c r="A50" t="inlineStr">
         <is>
           <t>BDRK_R0031</t>
@@ -4784,7 +4048,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -4793,7 +4057,7 @@
         </is>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51">
       <c r="A51" t="inlineStr">
         <is>
           <t>BDRK_R0004</t>
@@ -4801,7 +4065,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -4810,7 +4074,7 @@
         </is>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52">
       <c r="A52" t="inlineStr">
         <is>
           <t>BDRK_R0051</t>
@@ -4818,7 +4082,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -4827,7 +4091,7 @@
         </is>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53">
       <c r="A53" t="inlineStr">
         <is>
           <t>BDRK_R0046</t>
@@ -4835,7 +4099,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>BDRK_FBLK_IS_20260510_1000</t>
+          <t>BDRK_FBLK_IS______________</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -4913,7 +4177,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>BDRK_R0001</t>
@@ -4930,7 +4194,7 @@
         </is>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>BDRK_R0002</t>
@@ -4947,7 +4211,7 @@
         </is>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>BDRK_R0003</t>
@@ -4964,7 +4228,7 @@
         </is>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="inlineStr">
         <is>
           <t>BDRK_R0004</t>
@@ -4972,7 +4236,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000_AQ</t>
+          <t>BDRK_LBLK_IS_______________AQ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4981,7 +4245,7 @@
         </is>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" t="inlineStr">
         <is>
           <t>BDRK_R0005</t>
@@ -4998,7 +4262,7 @@
         </is>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="A7" t="inlineStr">
         <is>
           <t>BDRK_R0006</t>
@@ -5015,7 +4279,7 @@
         </is>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" t="inlineStr">
         <is>
           <t>BDRK_R0007</t>
@@ -5032,7 +4296,7 @@
         </is>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" t="inlineStr">
         <is>
           <t>BDRK_R0008</t>
@@ -5049,7 +4313,7 @@
         </is>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>BDRK_R0009</t>
@@ -5066,7 +4330,7 @@
         </is>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="A11" t="inlineStr">
         <is>
           <t>BDRK_R0010</t>
@@ -5083,7 +4347,7 @@
         </is>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12">
       <c r="A12" t="inlineStr">
         <is>
           <t>BDRK_R0011</t>
@@ -5100,7 +4364,7 @@
         </is>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13">
       <c r="A13" t="inlineStr">
         <is>
           <t>BDRK_R0012</t>
@@ -5117,7 +4381,7 @@
         </is>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14">
       <c r="A14" t="inlineStr">
         <is>
           <t>BDRK_R0013</t>
@@ -5134,7 +4398,7 @@
         </is>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15">
       <c r="A15" t="inlineStr">
         <is>
           <t>BDRK_R0014</t>
@@ -5151,7 +4415,7 @@
         </is>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16">
       <c r="A16" t="inlineStr">
         <is>
           <t>BDRK_R0015</t>
@@ -5168,7 +4432,7 @@
         </is>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17">
       <c r="A17" t="inlineStr">
         <is>
           <t>BDRK_R0016</t>
@@ -5185,7 +4449,7 @@
         </is>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18">
       <c r="A18" t="inlineStr">
         <is>
           <t>BDRK_R0017</t>
@@ -5202,7 +4466,7 @@
         </is>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19">
       <c r="A19" t="inlineStr">
         <is>
           <t>BDRK_R0018</t>
@@ -5219,7 +4483,7 @@
         </is>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20">
       <c r="A20" t="inlineStr">
         <is>
           <t>BDRK_R0019</t>
@@ -5236,7 +4500,7 @@
         </is>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21">
       <c r="A21" t="inlineStr">
         <is>
           <t>BDRK_R0020</t>
@@ -5253,7 +4517,7 @@
         </is>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22">
       <c r="A22" t="inlineStr">
         <is>
           <t>BDRK_R0021</t>
@@ -5270,7 +4534,7 @@
         </is>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23">
       <c r="A23" t="inlineStr">
         <is>
           <t>BDRK_R0022</t>
@@ -5287,7 +4551,7 @@
         </is>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24">
       <c r="A24" t="inlineStr">
         <is>
           <t>BDRK_R0023</t>
@@ -5304,7 +4568,7 @@
         </is>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25">
       <c r="A25" t="inlineStr">
         <is>
           <t>BDRK_R0024</t>
@@ -5321,7 +4585,7 @@
         </is>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26">
       <c r="A26" t="inlineStr">
         <is>
           <t>BDRK_R0025</t>
@@ -5338,7 +4602,7 @@
         </is>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27">
       <c r="A27" t="inlineStr">
         <is>
           <t>BDRK_R0026</t>
@@ -5355,7 +4619,7 @@
         </is>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28">
       <c r="A28" t="inlineStr">
         <is>
           <t>BDRK_R0027</t>
@@ -5372,7 +4636,7 @@
         </is>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29">
       <c r="A29" t="inlineStr">
         <is>
           <t>BDRK_R0028</t>
@@ -5389,7 +4653,7 @@
         </is>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30">
       <c r="A30" t="inlineStr">
         <is>
           <t>BDRK_R0029</t>
@@ -5406,7 +4670,7 @@
         </is>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31">
       <c r="A31" t="inlineStr">
         <is>
           <t>BDRK_R0030</t>
@@ -5423,7 +4687,7 @@
         </is>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32">
       <c r="A32" t="inlineStr">
         <is>
           <t>BDRK_R0031</t>
@@ -5431,7 +4695,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000_AQ</t>
+          <t>BDRK_LBLK_IS_______________AQ</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5440,7 +4704,7 @@
         </is>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33">
       <c r="A33" t="inlineStr">
         <is>
           <t>BDRK_R0032</t>
@@ -5457,7 +4721,7 @@
         </is>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34">
       <c r="A34" t="inlineStr">
         <is>
           <t>BDRK_R0033</t>
@@ -5474,7 +4738,7 @@
         </is>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35">
       <c r="A35" t="inlineStr">
         <is>
           <t>BDRK_R0034</t>
@@ -5491,7 +4755,7 @@
         </is>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36">
       <c r="A36" t="inlineStr">
         <is>
           <t>BDRK_R0035</t>
@@ -5508,7 +4772,7 @@
         </is>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37">
       <c r="A37" t="inlineStr">
         <is>
           <t>BDRK_R0036</t>
@@ -5525,7 +4789,7 @@
         </is>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38">
       <c r="A38" t="inlineStr">
         <is>
           <t>BDRK_R0037</t>
@@ -5542,7 +4806,7 @@
         </is>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39">
       <c r="A39" t="inlineStr">
         <is>
           <t>BDRK_R0038</t>
@@ -5559,7 +4823,7 @@
         </is>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40">
       <c r="A40" t="inlineStr">
         <is>
           <t>BDRK_R0039</t>
@@ -5576,7 +4840,7 @@
         </is>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41">
       <c r="A41" t="inlineStr">
         <is>
           <t>BDRK_R0040</t>
@@ -5593,7 +4857,7 @@
         </is>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42">
       <c r="A42" t="inlineStr">
         <is>
           <t>BDRK_R0041</t>
@@ -5610,7 +4874,7 @@
         </is>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43">
       <c r="A43" t="inlineStr">
         <is>
           <t>BDRK_R0042</t>
@@ -5627,7 +4891,7 @@
         </is>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44">
       <c r="A44" t="inlineStr">
         <is>
           <t>BDRK_R0043</t>
@@ -5644,7 +4908,7 @@
         </is>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45">
       <c r="A45" t="inlineStr">
         <is>
           <t>BDRK_R0044</t>
@@ -5661,7 +4925,7 @@
         </is>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46">
       <c r="A46" t="inlineStr">
         <is>
           <t>BDRK_R0045</t>
@@ -5678,7 +4942,7 @@
         </is>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47">
       <c r="A47" t="inlineStr">
         <is>
           <t>BDRK_R0046</t>
@@ -5686,7 +4950,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>BDRK_FBLK_IS_20260510_1000_AQ</t>
+          <t>BDRK_FBLK_IS_______________AQ</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5695,7 +4959,7 @@
         </is>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48">
       <c r="A48" t="inlineStr">
         <is>
           <t>BDRK_R0047</t>
@@ -5712,7 +4976,7 @@
         </is>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49">
       <c r="A49" t="inlineStr">
         <is>
           <t>BDRK_R0048</t>
@@ -5729,7 +4993,7 @@
         </is>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50">
       <c r="A50" t="inlineStr">
         <is>
           <t>BDRK_R0049</t>
@@ -5746,7 +5010,7 @@
         </is>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51">
       <c r="A51" t="inlineStr">
         <is>
           <t>BDRK_R0050</t>
@@ -5763,7 +5027,7 @@
         </is>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52">
       <c r="A52" t="inlineStr">
         <is>
           <t>BDRK_R0051</t>
@@ -5771,7 +5035,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000_AQ</t>
+          <t>BDRK_LBLK_IS_______________AQ</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -5780,7 +5044,7 @@
         </is>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53">
       <c r="A53" t="inlineStr">
         <is>
           <t>BDRK_R0052</t>
@@ -5797,7 +5061,7 @@
         </is>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54">
       <c r="A54" t="inlineStr">
         <is>
           <t>BDRK_R0001</t>
@@ -5814,7 +5078,7 @@
         </is>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55">
       <c r="A55" t="inlineStr">
         <is>
           <t>BDRK_R0002</t>
@@ -5831,7 +5095,7 @@
         </is>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56">
       <c r="A56" t="inlineStr">
         <is>
           <t>BDRK_R0003</t>
@@ -5848,7 +5112,7 @@
         </is>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57">
       <c r="A57" t="inlineStr">
         <is>
           <t>BDRK_R0004</t>
@@ -5856,7 +5120,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000_CN</t>
+          <t>BDRK_LBLK_IS_______________CN</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -5865,7 +5129,7 @@
         </is>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58">
       <c r="A58" t="inlineStr">
         <is>
           <t>BDRK_R0005</t>
@@ -5882,7 +5146,7 @@
         </is>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59">
       <c r="A59" t="inlineStr">
         <is>
           <t>BDRK_R0006</t>
@@ -5899,7 +5163,7 @@
         </is>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60">
       <c r="A60" t="inlineStr">
         <is>
           <t>BDRK_R0007</t>
@@ -5916,7 +5180,7 @@
         </is>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61">
       <c r="A61" t="inlineStr">
         <is>
           <t>BDRK_R0008</t>
@@ -5933,7 +5197,7 @@
         </is>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62">
       <c r="A62" t="inlineStr">
         <is>
           <t>BDRK_R0009</t>
@@ -5950,7 +5214,7 @@
         </is>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63">
       <c r="A63" t="inlineStr">
         <is>
           <t>BDRK_R0010</t>
@@ -5967,7 +5231,7 @@
         </is>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64">
       <c r="A64" t="inlineStr">
         <is>
           <t>BDRK_R0011</t>
@@ -5984,7 +5248,7 @@
         </is>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65">
       <c r="A65" t="inlineStr">
         <is>
           <t>BDRK_R0012</t>
@@ -6001,7 +5265,7 @@
         </is>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66">
       <c r="A66" t="inlineStr">
         <is>
           <t>BDRK_R0013</t>
@@ -6018,7 +5282,7 @@
         </is>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67">
       <c r="A67" t="inlineStr">
         <is>
           <t>BDRK_R0014</t>
@@ -6035,7 +5299,7 @@
         </is>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68">
       <c r="A68" t="inlineStr">
         <is>
           <t>BDRK_R0015</t>
@@ -6052,7 +5316,7 @@
         </is>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69">
       <c r="A69" t="inlineStr">
         <is>
           <t>BDRK_R0016</t>
@@ -6069,7 +5333,7 @@
         </is>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70">
       <c r="A70" t="inlineStr">
         <is>
           <t>BDRK_R0017</t>
@@ -6086,7 +5350,7 @@
         </is>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71">
       <c r="A71" t="inlineStr">
         <is>
           <t>BDRK_R0018</t>
@@ -6103,7 +5367,7 @@
         </is>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72">
       <c r="A72" t="inlineStr">
         <is>
           <t>BDRK_R0019</t>
@@ -6120,7 +5384,7 @@
         </is>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73">
       <c r="A73" t="inlineStr">
         <is>
           <t>BDRK_R0020</t>
@@ -6137,7 +5401,7 @@
         </is>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74">
       <c r="A74" t="inlineStr">
         <is>
           <t>BDRK_R0021</t>
@@ -6154,7 +5418,7 @@
         </is>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75">
       <c r="A75" t="inlineStr">
         <is>
           <t>BDRK_R0022</t>
@@ -6171,7 +5435,7 @@
         </is>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76">
       <c r="A76" t="inlineStr">
         <is>
           <t>BDRK_R0023</t>
@@ -6188,7 +5452,7 @@
         </is>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77">
       <c r="A77" t="inlineStr">
         <is>
           <t>BDRK_R0024</t>
@@ -6205,7 +5469,7 @@
         </is>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78">
       <c r="A78" t="inlineStr">
         <is>
           <t>BDRK_R0025</t>
@@ -6222,7 +5486,7 @@
         </is>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79">
       <c r="A79" t="inlineStr">
         <is>
           <t>BDRK_R0026</t>
@@ -6239,7 +5503,7 @@
         </is>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80">
       <c r="A80" t="inlineStr">
         <is>
           <t>BDRK_R0027</t>
@@ -6256,7 +5520,7 @@
         </is>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81">
       <c r="A81" t="inlineStr">
         <is>
           <t>BDRK_R0028</t>
@@ -6273,7 +5537,7 @@
         </is>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82">
       <c r="A82" t="inlineStr">
         <is>
           <t>BDRK_R0029</t>
@@ -6290,7 +5554,7 @@
         </is>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83">
       <c r="A83" t="inlineStr">
         <is>
           <t>BDRK_R0030</t>
@@ -6307,7 +5571,7 @@
         </is>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84">
       <c r="A84" t="inlineStr">
         <is>
           <t>BDRK_R0031</t>
@@ -6315,7 +5579,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000_CN</t>
+          <t>BDRK_LBLK_IS_______________CN</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -6324,7 +5588,7 @@
         </is>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85">
       <c r="A85" t="inlineStr">
         <is>
           <t>BDRK_R0032</t>
@@ -6341,7 +5605,7 @@
         </is>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86">
       <c r="A86" t="inlineStr">
         <is>
           <t>BDRK_R0033</t>
@@ -6358,7 +5622,7 @@
         </is>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87">
       <c r="A87" t="inlineStr">
         <is>
           <t>BDRK_R0034</t>
@@ -6375,7 +5639,7 @@
         </is>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88">
       <c r="A88" t="inlineStr">
         <is>
           <t>BDRK_R0035</t>
@@ -6392,7 +5656,7 @@
         </is>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89">
       <c r="A89" t="inlineStr">
         <is>
           <t>BDRK_R0036</t>
@@ -6409,7 +5673,7 @@
         </is>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90">
       <c r="A90" t="inlineStr">
         <is>
           <t>BDRK_R0037</t>
@@ -6426,7 +5690,7 @@
         </is>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91">
       <c r="A91" t="inlineStr">
         <is>
           <t>BDRK_R0038</t>
@@ -6443,7 +5707,7 @@
         </is>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92">
       <c r="A92" t="inlineStr">
         <is>
           <t>BDRK_R0039</t>
@@ -6460,7 +5724,7 @@
         </is>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93">
       <c r="A93" t="inlineStr">
         <is>
           <t>BDRK_R0040</t>
@@ -6477,7 +5741,7 @@
         </is>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94">
       <c r="A94" t="inlineStr">
         <is>
           <t>BDRK_R0041</t>
@@ -6494,7 +5758,7 @@
         </is>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95">
       <c r="A95" t="inlineStr">
         <is>
           <t>BDRK_R0042</t>
@@ -6511,7 +5775,7 @@
         </is>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96">
       <c r="A96" t="inlineStr">
         <is>
           <t>BDRK_R0043</t>
@@ -6528,7 +5792,7 @@
         </is>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97">
       <c r="A97" t="inlineStr">
         <is>
           <t>BDRK_R0044</t>
@@ -6545,7 +5809,7 @@
         </is>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98">
       <c r="A98" t="inlineStr">
         <is>
           <t>BDRK_R0045</t>
@@ -6562,7 +5826,7 @@
         </is>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99">
       <c r="A99" t="inlineStr">
         <is>
           <t>BDRK_R0046</t>
@@ -6570,7 +5834,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>BDRK_FBLK_IS_20260510_1000_CN</t>
+          <t>BDRK_FBLK_IS_______________CN</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -6579,7 +5843,7 @@
         </is>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100">
       <c r="A100" t="inlineStr">
         <is>
           <t>BDRK_R0047</t>
@@ -6596,7 +5860,7 @@
         </is>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101">
       <c r="A101" t="inlineStr">
         <is>
           <t>BDRK_R0048</t>
@@ -6613,7 +5877,7 @@
         </is>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102">
       <c r="A102" t="inlineStr">
         <is>
           <t>BDRK_R0049</t>
@@ -6630,7 +5894,7 @@
         </is>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103">
       <c r="A103" t="inlineStr">
         <is>
           <t>BDRK_R0050</t>
@@ -6647,7 +5911,7 @@
         </is>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104">
       <c r="A104" t="inlineStr">
         <is>
           <t>BDRK_R0051</t>
@@ -6655,7 +5919,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000_CN</t>
+          <t>BDRK_LBLK_IS_______________CN</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6664,7 +5928,7 @@
         </is>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105">
       <c r="A105" t="inlineStr">
         <is>
           <t>BDRK_R0052</t>
@@ -6768,7 +6032,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E500"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -6861,7 +6125,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C6" s="3"/>
@@ -7266,7 +6530,7 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C33" s="2"/>
@@ -7491,7 +6755,7 @@
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>BDRK_FBLK_IS_20260510_1000</t>
+          <t>BDRK_FBLK_IS______________</t>
         </is>
       </c>
       <c r="C48" s="3"/>
@@ -7566,7 +6830,7 @@
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C53" s="2"/>
@@ -7588,6 +6852,452 @@
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
     </row>
+    <row r="55" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="201" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="202" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="203" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="204" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="205" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="206" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="207" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="208" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="209" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="210" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="212" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="213" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="216" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="217" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="218" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="223" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="224" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="225" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="226" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="227" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="228" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="230" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="231" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="232" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="233" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="234" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="235" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="237" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="239" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="240" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="241" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="243" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="244" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="245" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="246" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="247" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="248" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="249" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="250" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="251" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="252" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="253" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="254" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="255" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="256" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="257" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="258" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="259" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="260" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="261" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="262" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="263" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="264" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="265" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="266" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="267" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="268" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="269" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="270" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="271" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="272" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="273" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="274" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="275" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="276" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="277" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="278" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="279" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="280" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="281" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="282" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="283" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="284" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="285" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="286" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="287" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="288" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="289" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="290" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="291" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="292" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="293" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="294" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="295" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="296" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="297" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="298" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="299" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="300" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="301" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="302" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="303" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="304" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="305" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="306" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="307" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="308" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="309" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="310" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="311" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="312" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="313" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="314" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="315" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="316" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="317" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="318" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="319" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="320" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="321" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="322" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="323" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="324" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="325" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="326" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="327" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="328" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="329" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="330" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="331" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="332" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="333" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="334" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="335" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="336" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="337" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="338" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="339" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="340" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="341" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="342" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="343" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="344" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="345" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="346" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="347" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="348" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="349" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="350" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="351" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="352" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="353" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="354" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="355" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="356" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="357" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="358" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="359" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="360" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="361" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="362" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="363" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="364" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="365" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="366" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="367" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="368" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="369" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="370" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="371" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="372" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="373" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="374" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="375" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="376" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="377" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="378" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="379" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="380" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="381" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="382" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="383" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="384" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="385" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="386" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="387" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="388" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="389" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="390" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="391" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="392" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="393" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="394" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="395" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="396" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="397" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="398" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="399" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="400" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="401" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="402" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="403" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="404" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="405" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="406" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="407" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="408" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="409" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="410" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="411" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="412" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="413" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="414" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="415" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="416" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="417" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="418" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="419" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="420" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="421" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="422" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="423" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="424" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="425" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="426" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="427" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="428" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="429" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="430" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="431" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="432" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="433" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="434" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="435" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="436" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="437" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="438" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="439" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="440" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="441" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="442" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="443" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="444" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="445" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="446" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="447" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="448" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="449" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="450" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="451" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="452" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="453" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="454" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="455" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="456" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="457" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="458" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="459" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="460" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="461" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="462" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="463" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="464" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="465" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="466" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="467" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="468" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="469" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="470" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="471" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="472" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="473" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="474" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="475" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="476" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="477" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="478" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="479" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="480" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="481" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="482" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="483" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="484" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="485" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="486" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="487" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="488" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="489" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="490" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="491" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="492" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="493" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="494" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="495" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="496" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="497" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="498" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="499" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="500" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="C1:D1"/>
@@ -7608,7 +7318,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H500"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" customWidth="1"/>
@@ -7732,7 +7442,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C6" s="3"/>
@@ -8218,7 +7928,7 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C33" s="4"/>
@@ -8488,7 +8198,7 @@
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>BDRK_FBLK_IS_20260510_1000</t>
+          <t>BDRK_FBLK_IS______________</t>
         </is>
       </c>
       <c r="C48" s="3"/>
@@ -8578,7 +8288,7 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C53" s="4"/>
@@ -8826,6 +8536,430 @@
       <c r="G76" s="3"/>
       <c r="H76" s="3"/>
     </row>
+    <row r="77" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="201" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="202" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="203" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="204" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="205" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="206" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="207" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="208" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="209" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="210" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="212" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="213" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="216" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="217" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="218" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="223" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="224" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="225" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="226" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="227" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="228" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="230" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="231" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="232" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="233" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="234" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="235" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="237" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="239" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="240" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="241" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="243" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="244" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="245" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="246" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="247" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="248" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="249" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="250" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="251" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="252" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="253" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="254" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="255" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="256" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="257" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="258" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="259" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="260" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="261" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="262" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="263" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="264" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="265" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="266" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="267" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="268" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="269" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="270" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="271" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="272" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="273" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="274" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="275" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="276" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="277" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="278" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="279" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="280" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="281" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="282" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="283" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="284" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="285" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="286" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="287" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="288" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="289" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="290" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="291" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="292" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="293" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="294" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="295" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="296" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="297" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="298" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="299" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="300" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="301" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="302" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="303" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="304" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="305" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="306" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="307" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="308" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="309" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="310" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="311" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="312" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="313" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="314" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="315" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="316" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="317" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="318" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="319" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="320" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="321" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="322" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="323" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="324" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="325" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="326" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="327" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="328" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="329" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="330" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="331" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="332" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="333" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="334" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="335" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="336" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="337" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="338" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="339" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="340" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="341" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="342" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="343" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="344" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="345" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="346" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="347" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="348" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="349" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="350" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="351" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="352" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="353" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="354" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="355" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="356" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="357" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="358" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="359" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="360" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="361" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="362" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="363" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="364" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="365" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="366" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="367" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="368" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="369" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="370" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="371" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="372" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="373" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="374" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="375" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="376" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="377" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="378" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="379" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="380" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="381" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="382" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="383" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="384" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="385" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="386" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="387" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="388" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="389" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="390" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="391" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="392" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="393" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="394" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="395" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="396" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="397" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="398" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="399" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="400" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="401" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="402" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="403" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="404" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="405" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="406" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="407" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="408" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="409" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="410" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="411" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="412" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="413" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="414" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="415" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="416" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="417" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="418" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="419" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="420" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="421" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="422" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="423" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="424" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="425" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="426" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="427" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="428" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="429" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="430" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="431" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="432" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="433" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="434" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="435" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="436" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="437" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="438" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="439" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="440" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="441" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="442" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="443" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="444" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="445" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="446" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="447" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="448" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="449" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="450" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="451" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="452" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="453" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="454" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="455" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="456" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="457" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="458" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="459" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="460" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="461" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="462" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="463" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="464" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="465" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="466" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="467" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="468" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="469" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="470" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="471" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="472" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="473" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="474" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="475" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="476" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="477" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="478" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="479" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="480" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="481" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="482" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="483" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="484" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="485" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="486" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="487" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="488" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="489" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="490" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="491" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="492" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="493" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="494" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="495" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="496" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="497" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="498" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="499" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="500" spans="1:8" ht="15.75" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
@@ -8845,7 +8979,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E500"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -8938,7 +9072,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C6" s="3"/>
@@ -9343,7 +9477,7 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C33" s="2"/>
@@ -9568,7 +9702,7 @@
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>BDRK_FBLK_IS_20260510_1000</t>
+          <t>BDRK_FBLK_IS______________</t>
         </is>
       </c>
       <c r="C48" s="3"/>
@@ -9643,14 +9777,460 @@
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>BDRK_LBLK_IS_20260510_1000</t>
+          <t>BDRK_LBLK_IS______________</t>
         </is>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
     </row>
-    <row r="54"/>
+    <row r="54" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="201" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="202" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="203" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="204" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="205" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="206" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="207" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="208" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="209" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="210" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="212" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="213" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="216" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="217" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="218" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="223" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="224" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="225" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="226" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="227" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="228" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="230" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="231" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="232" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="233" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="234" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="235" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="237" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="239" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="240" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="241" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="243" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="244" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="245" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="246" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="247" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="248" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="249" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="250" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="251" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="252" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="253" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="254" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="255" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="256" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="257" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="258" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="259" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="260" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="261" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="262" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="263" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="264" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="265" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="266" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="267" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="268" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="269" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="270" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="271" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="272" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="273" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="274" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="275" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="276" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="277" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="278" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="279" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="280" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="281" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="282" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="283" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="284" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="285" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="286" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="287" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="288" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="289" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="290" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="291" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="292" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="293" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="294" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="295" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="296" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="297" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="298" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="299" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="300" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="301" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="302" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="303" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="304" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="305" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="306" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="307" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="308" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="309" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="310" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="311" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="312" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="313" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="314" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="315" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="316" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="317" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="318" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="319" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="320" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="321" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="322" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="323" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="324" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="325" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="326" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="327" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="328" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="329" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="330" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="331" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="332" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="333" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="334" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="335" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="336" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="337" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="338" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="339" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="340" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="341" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="342" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="343" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="344" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="345" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="346" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="347" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="348" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="349" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="350" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="351" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="352" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="353" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="354" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="355" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="356" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="357" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="358" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="359" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="360" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="361" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="362" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="363" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="364" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="365" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="366" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="367" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="368" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="369" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="370" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="371" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="372" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="373" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="374" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="375" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="376" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="377" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="378" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="379" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="380" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="381" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="382" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="383" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="384" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="385" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="386" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="387" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="388" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="389" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="390" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="391" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="392" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="393" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="394" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="395" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="396" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="397" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="398" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="399" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="400" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="401" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="402" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="403" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="404" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="405" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="406" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="407" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="408" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="409" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="410" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="411" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="412" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="413" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="414" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="415" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="416" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="417" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="418" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="419" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="420" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="421" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="422" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="423" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="424" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="425" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="426" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="427" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="428" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="429" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="430" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="431" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="432" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="433" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="434" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="435" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="436" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="437" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="438" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="439" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="440" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="441" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="442" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="443" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="444" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="445" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="446" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="447" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="448" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="449" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="450" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="451" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="452" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="453" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="454" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="455" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="456" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="457" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="458" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="459" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="460" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="461" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="462" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="463" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="464" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="465" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="466" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="467" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="468" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="469" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="470" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="471" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="472" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="473" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="474" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="475" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="476" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="477" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="478" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="479" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="480" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="481" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="482" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="483" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="484" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="485" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="486" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="487" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="488" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="489" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="490" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="491" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="492" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="493" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="494" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="495" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="496" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="497" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="498" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="499" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="500" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="C1:D1"/>

</xml_diff>